<commit_message>
Carry the pack's line commentary beside the Financial Summary
The CIB page sets a short note against each line - MSS, GPS, GTS, C&L, ECL,
Direct Costs, Deposits, L&A - and the app had nowhere to put them: driver
notes only surfaced as a lead sentence in the generated commentary.

The Financial Summary now prints the column beneath the grid. A note written
by the business leads, from the Drivers pane or the config's Drivers sheet
keyed by the line name; a line without one reads its own figures in the
page's own movement wording and in that line's own unit, so the note and the
row beside it cannot disagree. fsum_note_lines sets which lines are
commented and in what order, fsum_notes turns the column on or off, and the
Word export carries it.

The CIB config lists the pack's own commented lines in the pack's order.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01P4DDZgm6WRNJpLjFRThM8B
</commit_message>
<xml_diff>
--- a/iwpb-sg-dashboard/CIB_dashboard_config_pack.xlsx
+++ b/iwpb-sg-dashboard/CIB_dashboard_config_pack.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B26"/>
+  <dimension ref="A1:B28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -737,10 +737,34 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
+          <t>fsum_notes</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>fsum_note_lines</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>MSS;Global Payments Solutions;Global Trade Solutions;Credit and Lending;HIF;CMA Net;Other Revenue;ECLs (ex Notables);Direct Costs (ex VP);Variable Pay (VP);Indirect Costs;Customers and Banks Deposits (PE);Loans and Advances to Customers and Banks (PE)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
           <t>show_greeting</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="B28" t="inlineStr">
         <is>
           <t>N</t>
         </is>

</xml_diff>

<commit_message>
Let the config file own the disclaimer's wording
commentary_disclaimer was already read from the Settings sheet, but neither
the repo's config CSV nor the two worked packs carried the row, so nobody
could see it was theirs to set. The CSV now lists every current commentary
setting (the disclaimer, style, clause cap, driver floor/cover, note cap),
both packs are rebuilt from it, and the CIB pack sets its own wording as a
worked example — check_cfgdisc.js proves the config's words reach the page
and the Word export alike. Leaving the row out keeps the standard text.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01P4DDZgm6WRNJpLjFRThM8B
</commit_message>
<xml_diff>
--- a/iwpb-sg-dashboard/CIB_dashboard_config_pack.xlsx
+++ b/iwpb-sg-dashboard/CIB_dashboard_config_pack.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B28"/>
+  <dimension ref="A1:B29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -749,22 +749,34 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>fsum_note_lines</t>
+          <t>commentary_disclaimer</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>MSS;Global Payments Solutions;Global Trade Solutions;Credit and Lending;HIF;CMA Net;Other Revenue;ECLs (ex Notables);Direct Costs (ex VP);Variable Pay (VP);Indirect Costs;Customers and Banks Deposits (PE);Loans and Advances to Customers and Banks (PE)</t>
+          <t>This CIB Asia &amp; MENAT commentary has been generated from the figures in the file and the commentary document loaded with it. It may be inaccurate and/or incomplete. Review and edit before further use or distribution.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
+          <t>fsum_note_lines</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>MSS;Global Payments Solutions;Global Trade Solutions;Credit and Lending;HIF;CMA Net;Other Revenue;ECLs (ex Notables);Direct Costs (ex VP);Variable Pay (VP);Indirect Costs;Customers and Banks Deposits (PE);Loans and Advances to Customers and Banks (PE)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
           <t>show_greeting</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
+      <c r="B29" t="inlineStr">
         <is>
           <t>N</t>
         </is>

</xml_diff>

<commit_message>
No Commentary tab in the driller; the words live in the configuration
The driller carries figures only. Its Commentary-tab reading is removed —
a tab by that name is still never parsed as data, simply ignored — and the
one way written commentary arrives is the configuration's Commentary section,
which now also accepts bare paragraphs: unstructured commentary, matched
against whatever names the loaded driller carries, exactly as the tab's
paragraphs were. Addressed rows (View | Line | Text) are unchanged.

The worked commentary moves accordingly: the IWPB pack's Commentary sheet
carries the eight untagged paragraphs, the CIB pack's carries five addressed
rows, the six-basis driller loses its tab, the withCommentary driller sample
is removed, and the six-basis Word download is regenerated from driller plus
pack.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01P4DDZgm6WRNJpLjFRThM8B
</commit_message>
<xml_diff>
--- a/iwpb-sg-dashboard/CIB_dashboard_config_pack.xlsx
+++ b/iwpb-sg-dashboard/CIB_dashboard_config_pack.xlsx
@@ -14,10 +14,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Views" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Labels" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Drivers" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metrics" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ProductHierarchy" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AccountHierarchy" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CountryHierarchy" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Commentary" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metrics" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ProductHierarchy" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AccountHierarchy" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CountryHierarchy" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -793,6 +794,816 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:G31"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Level 1</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Level 2</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Level 3</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Level 4</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Level 5</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Match</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>B1</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>CIB</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>B2</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>CIB</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Markets and Securities Services</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>B3</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>CIB</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Markets and Securities Services</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Markets</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>B4</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>CIB</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Markets and Securities Services</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Markets</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Foreign Exchange</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Foreign Exchange|FX</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>B5</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>CIB</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Markets and Securities Services</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Markets</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Rates</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Rates</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>B6</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>CIB</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Markets and Securities Services</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Markets</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Credit Trading</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>B7</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>CIB</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Markets and Securities Services</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Markets</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Equities</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Equities</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>B8</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>CIB</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Markets and Securities Services</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Securities Services</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>B9</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>CIB</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Markets and Securities Services</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Securities Services</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Custody</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Custody</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>B10</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>CIB</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Markets and Securities Services</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Securities Services</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Fund Administration</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Fund Administration</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>B11</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>CIB</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Markets and Securities Services</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Securities Services</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Issuer Services</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Issuer Services</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>B12</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>CIB</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Global Payments Solutions</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>B13</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>CIB</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Global Payments Solutions</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Payments and Cash Management</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Payments and Cash Management|PCM</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>B14</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>CIB</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Global Payments Solutions</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Liquidity Management</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Liquidity Management</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>B15</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>CIB</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Global Payments Solutions</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Commercial Cards</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Commercial Cards</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>B16</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>CIB</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Global Trade Solutions</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>B17</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>CIB</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Global Trade Solutions</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Documentary Trade</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Documentary Trade</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>B18</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>CIB</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Global Trade Solutions</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Receivables Finance</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Receivables Finance</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>B19</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>CIB</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Global Trade Solutions</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Guarantees</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Guarantees</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>B20</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>CIB</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Credit and Lending</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>B21</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>CIB</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Credit and Lending</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Corporate Lending</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Corporate Lending</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>B22</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>CIB</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Credit and Lending</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Structured Finance</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Structured Finance</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>B23</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>CIB</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Credit and Lending</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Portfolio Management</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Portfolio Management</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>B24</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>CIB</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Capital Markets and Advisory</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>B25</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>CIB</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Capital Markets and Advisory</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Debt Capital Markets</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Debt Capital Markets|DCM</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>B26</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>CIB</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Capital Markets and Advisory</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Equity Capital Markets</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Equity Capital Markets|ECM</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>B27</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>CIB</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Capital Markets and Advisory</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Advisory</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Advisory</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>B28</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>CIB</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>HIF</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>HIF</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>B29</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>CIB</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>B30</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Non product aligned</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Non product aligned</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:G34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1673,7 +2484,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2879,262 +3690,103 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B21"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="42" customWidth="1" min="1" max="1"/>
-    <col width="48" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="70" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Key</t>
+          <t>View</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Scope</t>
+          <t>Line</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Text</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Total Revenue (ex Notables)</t>
+          <t>Financial Summary</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>accH3=Total Revenue (ex Notables)</t>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Rates and FX carried the half; deposit margin narrowed broadly as planned.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>MSS</t>
+          <t>Chart</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>accH4=MSS</t>
+          <t>Markets and Securities Services</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Rates and FX led the half while Custody stayed soft.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Global Payments Solutions</t>
+          <t>Chart</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>accH4=Global Payments Solutions</t>
+          <t>Global Trade Solutions</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Drawdowns slipped into July - timing, not demand. The pipeline is intact.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Credit and Lending</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>accH4=Credit and Lending</t>
+          <t>Summary</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>June closes the half ahead of plan on revenue and behind on costs.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Global Trade Solutions</t>
-        </is>
-      </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>accH4=Global Trade Solutions</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>HIF</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>accH4=HIF</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>CMA Net</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>accH4=CMA Net</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Other Revenue</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>accH4=Other Revenue</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Banking NII</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>income=Banking NII</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Fee and other income</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>income=Fee and other income</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>ECLs (ex Notables)</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>accH3=ECLs (ex Notables)</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Direct Costs (ex VP)</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>accH4=Direct Costs (ex VP)</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Variable Pay (VP)</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>accH4=Variable Pay (VP)</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Indirect Costs</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>accH4=Indirect Costs</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Total Operating Expenses (ex Notables)</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>accH3=Total Operating Expenses (ex Notables)</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>PBT (ex Notables)</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>accH2=PBT (ex Notables)</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>PBT (Reported)</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>accH1=PBT (Reported)</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Customer Deposits (PE)</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>accH2=o/w Customer Deposits (PE)</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Loans and Advances to Customers (PE)</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>accH2=o/w Loans and Advances to Customers (PE)</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Total RWAs</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>accH1=Total RWAs</t>
+          <t>Global Payments Solutions</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Payments volumes held up well; liquidity margin thinner as rates came off.</t>
         </is>
       </c>
     </row>
@@ -3149,802 +3801,262 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G31"/>
+  <dimension ref="A1:B21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="34" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="26" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
-    <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="48" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>ID</t>
+          <t>Key</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Level 1</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Level 2</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Level 3</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Level 4</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Level 5</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Match</t>
+          <t>Scope</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>B1</t>
+          <t>Total Revenue (ex Notables)</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>CIB</t>
+          <t>accH3=Total Revenue (ex Notables)</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>B2</t>
+          <t>MSS</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>CIB</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Markets and Securities Services</t>
+          <t>accH4=MSS</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>B3</t>
+          <t>Global Payments Solutions</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>CIB</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Markets and Securities Services</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Markets</t>
+          <t>accH4=Global Payments Solutions</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>B4</t>
+          <t>Credit and Lending</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>CIB</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Markets and Securities Services</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Markets</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Foreign Exchange</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>Foreign Exchange|FX</t>
+          <t>accH4=Credit and Lending</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>B5</t>
+          <t>Global Trade Solutions</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>CIB</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Markets and Securities Services</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Markets</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>Rates</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>Rates</t>
+          <t>accH4=Global Trade Solutions</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>B6</t>
+          <t>HIF</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>CIB</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Markets and Securities Services</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Markets</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>Credit</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>Credit Trading</t>
+          <t>accH4=HIF</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>B7</t>
+          <t>CMA Net</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>CIB</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Markets and Securities Services</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Markets</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>Equities</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>Equities</t>
+          <t>accH4=CMA Net</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>B8</t>
+          <t>Other Revenue</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>CIB</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Markets and Securities Services</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Securities Services</t>
+          <t>accH4=Other Revenue</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>B9</t>
+          <t>Banking NII</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>CIB</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Markets and Securities Services</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Securities Services</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>Custody</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>Custody</t>
+          <t>income=Banking NII</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>B10</t>
+          <t>Fee and other income</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>CIB</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Markets and Securities Services</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>Securities Services</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>Fund Administration</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>Fund Administration</t>
+          <t>income=Fee and other income</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>B11</t>
+          <t>ECLs (ex Notables)</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>CIB</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Markets and Securities Services</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>Securities Services</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>Issuer Services</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>Issuer Services</t>
+          <t>accH3=ECLs (ex Notables)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>B12</t>
+          <t>Direct Costs (ex VP)</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>CIB</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Global Payments Solutions</t>
+          <t>accH4=Direct Costs (ex VP)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>B13</t>
+          <t>Variable Pay (VP)</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>CIB</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Global Payments Solutions</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>Payments and Cash Management</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>Payments and Cash Management|PCM</t>
+          <t>accH4=Variable Pay (VP)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>B14</t>
+          <t>Indirect Costs</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>CIB</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>Global Payments Solutions</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>Liquidity Management</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>Liquidity Management</t>
+          <t>accH4=Indirect Costs</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>B15</t>
+          <t>Total Operating Expenses (ex Notables)</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>CIB</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>Global Payments Solutions</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>Commercial Cards</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>Commercial Cards</t>
+          <t>accH3=Total Operating Expenses (ex Notables)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>B16</t>
+          <t>PBT (ex Notables)</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>CIB</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>Global Trade Solutions</t>
+          <t>accH2=PBT (ex Notables)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>B17</t>
+          <t>PBT (Reported)</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>CIB</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>Global Trade Solutions</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>Documentary Trade</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>Documentary Trade</t>
+          <t>accH1=PBT (Reported)</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>B18</t>
+          <t>Customer Deposits (PE)</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>CIB</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>Global Trade Solutions</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>Receivables Finance</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>Receivables Finance</t>
+          <t>accH2=o/w Customer Deposits (PE)</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>B19</t>
+          <t>Loans and Advances to Customers (PE)</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>CIB</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>Global Trade Solutions</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>Guarantees</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>Guarantees</t>
+          <t>accH2=o/w Loans and Advances to Customers (PE)</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>B20</t>
+          <t>Total RWAs</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>CIB</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>Credit and Lending</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>B21</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>CIB</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>Credit and Lending</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>Corporate Lending</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>Corporate Lending</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>B22</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>CIB</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>Credit and Lending</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>Structured Finance</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>Structured Finance</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>B23</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>CIB</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>Credit and Lending</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>Portfolio Management</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>Portfolio Management</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>B24</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>CIB</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>Capital Markets and Advisory</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>B25</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>CIB</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>Capital Markets and Advisory</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>Debt Capital Markets</t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>Debt Capital Markets|DCM</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>B26</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>CIB</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>Capital Markets and Advisory</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>Equity Capital Markets</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>Equity Capital Markets|ECM</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>B27</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>CIB</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>Capital Markets and Advisory</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>Advisory</t>
-        </is>
-      </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>Advisory</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>B28</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>CIB</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>HIF</t>
-        </is>
-      </c>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>HIF</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>B29</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>CIB</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>Other</t>
-        </is>
-      </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>Other</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>B30</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>Non product aligned</t>
-        </is>
-      </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>Non product aligned</t>
+          <t>accH1=Total RWAs</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
The configuration decides which tiles show
tile_hidden parks the tiles it names - exact names or patterns matched
against the whole name, so cost.* parks every cost line - and a new
tile_visible keeps only the named tiles and parks the rest. Parked
tiles stay one click away behind the Show parked strip, the reader's
own show/hide toggle still wins on their screen (kept as a restore
even against a pattern or the show-list), and uploading a
configuration re-baselines the tiles so its policy is not shadowed by
toggles made under the previous one. Both packs and the CSV surface
the two settings.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01P4DDZgm6WRNJpLjFRThM8B
</commit_message>
<xml_diff>
--- a/iwpb-sg-dashboard/CIB_dashboard_config_pack.xlsx
+++ b/iwpb-sg-dashboard/CIB_dashboard_config_pack.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B31"/>
+  <dimension ref="A1:B32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -817,6 +817,14 @@
           <t>auto</t>
         </is>
       </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>tile_visible</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3467,7 +3475,6 @@
           <t>Exec brief</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr">
         <is>
           <t>{line} {var} {vs}, led by {drivers}.</t>
@@ -3480,7 +3487,6 @@
           <t>FP&amp;A detail</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr">
         <is>
           <t>{line}: {main} against {base} — {varamt} ({varpct}) {vs}. Key movers: {drivers}.</t>
@@ -3493,8 +3499,6 @@
           <t>&lt;i&gt;Scope words: Group · Global · Regional · Country, optionally led by a business (IWPB Global) or a place (Singapore). With the style set to Auto — match the scope, the page adopts the best-fitting template as the scope moves; no scoped template defined for a scope means the pack narrative speaks there. A blank scope makes a named style picked by hand.</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
-      <c r="C8" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
The file being loaded is a TM1 extract, not a driller file
- Ingest page heading, drop zone, upload text and the left-pane button all
  read Ingest TM1 Extract; the heading and drop zone gain label keys
  (ingest_title, ingest_drop) so the wording stays config-driven
- Parse errors, the MI assistant's replies and the config templates name
  the TM1 extract too, so one vocabulary runs through the page
- Labels sheet updated in the Group, IWPB and CIB packs
- README + docx follow, leaving sample filenames and the product name
  untouched

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01P4DDZgm6WRNJpLjFRThM8B
</commit_message>
<xml_diff>
--- a/iwpb-sg-dashboard/CIB_dashboard_config_pack.xlsx
+++ b/iwpb-sg-dashboard/CIB_dashboard_config_pack.xlsx
@@ -824,7 +824,6 @@
           <t>tile_visible</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3772,7 +3771,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3824,6 +3823,30 @@
       <c r="B4" t="inlineStr">
         <is>
           <t>KPIs · CIB lines</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>ingest_title</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Ingest TM1 Extract</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>ingest_drop</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Drop the TM1 extract here</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tile size comes from the configuration
tile_height sets the height every tile shares and tile_min_width sets the
narrowest a tile may become before the grid drops a column, so a pack can
make the summary roomier or fit more tiles per row without touching the
page. Both are registered settings, so they reach the downloadable
template, and unusable values fall back rather than breaking the grid.

Also fixes a doubled word the TM1 rename left in the README opening.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01P4DDZgm6WRNJpLjFRThM8B
</commit_message>
<xml_diff>
--- a/iwpb-sg-dashboard/CIB_dashboard_config_pack.xlsx
+++ b/iwpb-sg-dashboard/CIB_dashboard_config_pack.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B32"/>
+  <dimension ref="A1:B34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -823,6 +823,26 @@
         <is>
           <t>tile_visible</t>
         </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>tile_height</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>tile_min_width</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>236</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
The left rail reads in one case, and a pack can word every entry
Business performance and All commentaries were the odd two out in the rail:
nav_bizperf had no default at all and nav_comall's was worded unlike its
siblings, so a pack that titles its navigation left those two in another
case. Both now have defaults in step with the rest, the built-in wording is
Title Case throughout, and the three packs carry explicit rows so they keep
their own sentence-case house style.

Reverts the page-heading case change from the previous commit — the request
was about the rail, and those headings match the other pages as they were.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01P4DDZgm6WRNJpLjFRThM8B
</commit_message>
<xml_diff>
--- a/iwpb-sg-dashboard/CIB_dashboard_config_pack.xlsx
+++ b/iwpb-sg-dashboard/CIB_dashboard_config_pack.xlsx
@@ -3791,7 +3791,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3867,6 +3867,30 @@
       <c r="B6" t="inlineStr">
         <is>
           <t>Drop the TM1 extract here</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>nav_bizperf</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Business performance</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>nav_comall</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>All commentaries</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
The ingest action is named Ingest TM1 Data Extract
The left-pane button, the page it opens and the drop zone all name the same
action, so all three carry the new wording, in the app's defaults and in the
Group, IWPB and CIB packs. CIB had no btn_newfile row and was inheriting the
default; it now carries one like the others.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01P4DDZgm6WRNJpLjFRThM8B
</commit_message>
<xml_diff>
--- a/iwpb-sg-dashboard/CIB_dashboard_config_pack.xlsx
+++ b/iwpb-sg-dashboard/CIB_dashboard_config_pack.xlsx
@@ -3791,7 +3791,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3854,7 +3854,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Ingest TM1 Extract</t>
+          <t>Ingest TM1 Data Extract</t>
         </is>
       </c>
     </row>
@@ -3866,7 +3866,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Drop the TM1 extract here</t>
+          <t>Drop the TM1 data extract here</t>
         </is>
       </c>
     </row>
@@ -3891,6 +3891,18 @@
       <c r="B8" t="inlineStr">
         <is>
           <t>All commentaries</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>btn_newfile</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Ingest TM1 Data Extract</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
The left pane is worded entirely from the configuration
Every heading and label in the rail was already bound to a key, but the
control surface was incomplete and partly fictional: sect_comtpl, lbl_year
and lbl_tplpick reached no pack, the CIB pack carried one label row, and
sect_kpis, sect_filters, sect_output and nav_table were offered in the
template and the packs while nothing on the page read them.

The defaults now hold only keys the page consumes, and all three packs carry
that exact set with their own wording preserved, so a row in the Labels sheet
always does something and every heading in the pane can be renamed from it.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01P4DDZgm6WRNJpLjFRThM8B
</commit_message>
<xml_diff>
--- a/iwpb-sg-dashboard/CIB_dashboard_config_pack.xlsx
+++ b/iwpb-sg-dashboard/CIB_dashboard_config_pack.xlsx
@@ -45,7 +45,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -55,6 +55,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00DB0011"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="009E1B32"/>
       </patternFill>
     </fill>
   </fills>
@@ -70,10 +75,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -3791,20 +3797,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="46" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>Key</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
@@ -3825,84 +3831,300 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>nav_fsum</t>
+          <t>nav_custom</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Financial Summary</t>
+          <t>My dashboard</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>sect_kpis</t>
+          <t>nav_builder</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>KPIs · CIB lines</t>
+          <t>Drag &amp; drop charts</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ingest_title</t>
+          <t>nav_query</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Ingest TM1 Data Extract</t>
+          <t>Query builder</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ingest_drop</t>
+          <t>nav_assist</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Drop the TM1 data extract here</t>
+          <t>MI Assistant</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>nav_bizperf</t>
+          <t>nav_sim</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Business performance</t>
+          <t>Simulation Assistant</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>nav_comall</t>
+          <t>nav_fsum</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>All commentaries</t>
+          <t>Financial Summary</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>nav_comall</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>All commentaries</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>nav_bizperf</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Business performance</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>sect_dashboards</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>KPI Dashboards</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>sect_config</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Configuration</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>sect_period</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Period</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>sect_comtpl</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Commentary templates</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
           <t>btn_newfile</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B15" t="inlineStr">
         <is>
           <t>Ingest TM1 Data Extract</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>ingest_title</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Ingest TM1 Data Extract</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>ingest_drop</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Drop the TM1 data extract here</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>btn_regen</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Regenerate</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>btn_retrieve</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Retrieve</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>lbl_year</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>lbl_ytd</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>YTD through</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>lbl_varper</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Variance period</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>lbl_units</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Units</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>lbl_scope</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Scope</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>lbl_tplpick</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Active style</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>dec_eyebrow</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Decisions required</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>dec_title</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Executive decisions</t>
         </is>
       </c>
     </row>

</xml_diff>